<commit_message>
Excel: fix invalid defined names that Excel stripped on open
Excel reported repaired named ranges and removed formulas in Geometry,
Stress and Pressure. Cause: the defined name "Rc" equals the R1C1
reference notation RC, so Excel rejected it and dropped every formula
that used it (Rv, Rs renamed alongside; CC renamed preventively).
- RENAME map: Rc->R_crest, Rv->R_valley, Rs->R_sum, CC->C_ye
- check_name(): rejects A1-like, R1C1-like, bare R/C, TRUE/FALSE and
  malformed names at generation time; case-insensitive collision assert
- workbook regenerated and re-verified with the formulas evaluator
  (28 base items 1.5e-7, 8 pressure items 5.5e-4, no error cells);
  scan confirms no stale tokens and no non-ASCII outside string literals
- docs/10 and 03 updated

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HxmfvHAm4o1QfibMbn4i2r
</commit_message>
<xml_diff>
--- a/calc/SPHX_EQV_calc.xlsx
+++ b/calc/SPHX_EQV_calc.xlsx
@@ -57,7 +57,7 @@
     <definedName name="f_">'Geometry'!$B$12</definedName>
     <definedName name="Rc_in">'Geometry'!$B$16</definedName>
     <definedName name="Rv_in">'Geometry'!$B$17</definedName>
-    <definedName name="Rs">'Geometry'!$B$18</definedName>
+    <definedName name="R_sum">'Geometry'!$B$18</definedName>
     <definedName name="a_hi">'Geometry'!$B$19</definedName>
     <definedName name="alpha_A">'Geometry'!$B$44</definedName>
     <definedName name="resid_A">'Geometry'!$B$45</definedName>
@@ -65,8 +65,8 @@
     <definedName name="R_B">'Geometry'!$B$47</definedName>
     <definedName name="alpha">'Geometry'!$B$48</definedName>
     <definedName name="alpha_deg">'Geometry'!$B$49</definedName>
-    <definedName name="Rc">'Geometry'!$B$50</definedName>
-    <definedName name="Rv">'Geometry'!$B$51</definedName>
+    <definedName name="R_crest">'Geometry'!$B$50</definedName>
+    <definedName name="R_valley">'Geometry'!$B$51</definedName>
     <definedName name="TL">'Geometry'!$B$52</definedName>
     <definedName name="Rmin">'Geometry'!$B$53</definedName>
     <definedName name="chk_geom">'Geometry'!$B$54</definedName>
@@ -161,7 +161,7 @@
     <definedName name="kxx">'Stress'!$B$23</definedName>
     <definedName name="kyy">'Stress'!$B$24</definedName>
     <definedName name="kxy">'Stress'!$B$25</definedName>
-    <definedName name="CC">'Stress'!$B$29</definedName>
+    <definedName name="C_ye">'Stress'!$B$29</definedName>
     <definedName name="c_1">'Stress'!$B$30</definedName>
     <definedName name="c_4">'Stress'!$B$31</definedName>
     <definedName name="ch_c">'Stress'!$B$32</definedName>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>MIN(ASIN(MIN(1,c_/Rs)),ACOS(MAX(-1,1-H_mid/Rs)),PI()/2)-0.000001</f>
+        <f>MIN(ASIN(MIN(1,c_/R_sum)),ACOS(MAX(-1,1-H_mid/R_sum)),PI()/2)-0.000001</f>
         <v/>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -2204,15 +2204,15 @@
         <v>0</v>
       </c>
       <c r="B22" s="15">
-        <f>MIN(a_hi,MAX(0.001,ATAN(H_mid/MAX(c_-Rs*0.5,0.001))))</f>
+        <f>MIN(a_hi,MAX(0.001,ATAN(H_mid/MAX(c_-R_sum*0.5,0.001))))</f>
         <v/>
       </c>
       <c r="C22" s="16">
-        <f>Rs*(1-COS($B$22))+(c_-Rs*SIN($B$22))*TAN($B$22)-H_mid</f>
+        <f>R_sum*(1-COS($B$22))+(c_-R_sum*SIN($B$22))*TAN($B$22)-H_mid</f>
         <v/>
       </c>
       <c r="D22" s="15">
-        <f>(c_-Rs*SIN($B$22))/COS($B$22)^2</f>
+        <f>(c_-R_sum*SIN($B$22))/COS($B$22)^2</f>
         <v/>
       </c>
     </row>
@@ -2225,11 +2225,11 @@
         <v/>
       </c>
       <c r="C23" s="16">
-        <f>Rs*(1-COS($B$23))+(c_-Rs*SIN($B$23))*TAN($B$23)-H_mid</f>
+        <f>R_sum*(1-COS($B$23))+(c_-R_sum*SIN($B$23))*TAN($B$23)-H_mid</f>
         <v/>
       </c>
       <c r="D23" s="15">
-        <f>(c_-Rs*SIN($B$23))/COS($B$23)^2</f>
+        <f>(c_-R_sum*SIN($B$23))/COS($B$23)^2</f>
         <v/>
       </c>
     </row>
@@ -2242,11 +2242,11 @@
         <v/>
       </c>
       <c r="C24" s="16">
-        <f>Rs*(1-COS($B$24))+(c_-Rs*SIN($B$24))*TAN($B$24)-H_mid</f>
+        <f>R_sum*(1-COS($B$24))+(c_-R_sum*SIN($B$24))*TAN($B$24)-H_mid</f>
         <v/>
       </c>
       <c r="D24" s="15">
-        <f>(c_-Rs*SIN($B$24))/COS($B$24)^2</f>
+        <f>(c_-R_sum*SIN($B$24))/COS($B$24)^2</f>
         <v/>
       </c>
     </row>
@@ -2259,11 +2259,11 @@
         <v/>
       </c>
       <c r="C25" s="16">
-        <f>Rs*(1-COS($B$25))+(c_-Rs*SIN($B$25))*TAN($B$25)-H_mid</f>
+        <f>R_sum*(1-COS($B$25))+(c_-R_sum*SIN($B$25))*TAN($B$25)-H_mid</f>
         <v/>
       </c>
       <c r="D25" s="15">
-        <f>(c_-Rs*SIN($B$25))/COS($B$25)^2</f>
+        <f>(c_-R_sum*SIN($B$25))/COS($B$25)^2</f>
         <v/>
       </c>
     </row>
@@ -2276,11 +2276,11 @@
         <v/>
       </c>
       <c r="C26" s="16">
-        <f>Rs*(1-COS($B$26))+(c_-Rs*SIN($B$26))*TAN($B$26)-H_mid</f>
+        <f>R_sum*(1-COS($B$26))+(c_-R_sum*SIN($B$26))*TAN($B$26)-H_mid</f>
         <v/>
       </c>
       <c r="D26" s="15">
-        <f>(c_-Rs*SIN($B$26))/COS($B$26)^2</f>
+        <f>(c_-R_sum*SIN($B$26))/COS($B$26)^2</f>
         <v/>
       </c>
     </row>
@@ -2293,11 +2293,11 @@
         <v/>
       </c>
       <c r="C27" s="16">
-        <f>Rs*(1-COS($B$27))+(c_-Rs*SIN($B$27))*TAN($B$27)-H_mid</f>
+        <f>R_sum*(1-COS($B$27))+(c_-R_sum*SIN($B$27))*TAN($B$27)-H_mid</f>
         <v/>
       </c>
       <c r="D27" s="15">
-        <f>(c_-Rs*SIN($B$27))/COS($B$27)^2</f>
+        <f>(c_-R_sum*SIN($B$27))/COS($B$27)^2</f>
         <v/>
       </c>
     </row>
@@ -2310,11 +2310,11 @@
         <v/>
       </c>
       <c r="C28" s="16">
-        <f>Rs*(1-COS($B$28))+(c_-Rs*SIN($B$28))*TAN($B$28)-H_mid</f>
+        <f>R_sum*(1-COS($B$28))+(c_-R_sum*SIN($B$28))*TAN($B$28)-H_mid</f>
         <v/>
       </c>
       <c r="D28" s="15">
-        <f>(c_-Rs*SIN($B$28))/COS($B$28)^2</f>
+        <f>(c_-R_sum*SIN($B$28))/COS($B$28)^2</f>
         <v/>
       </c>
     </row>
@@ -2327,11 +2327,11 @@
         <v/>
       </c>
       <c r="C29" s="16">
-        <f>Rs*(1-COS($B$29))+(c_-Rs*SIN($B$29))*TAN($B$29)-H_mid</f>
+        <f>R_sum*(1-COS($B$29))+(c_-R_sum*SIN($B$29))*TAN($B$29)-H_mid</f>
         <v/>
       </c>
       <c r="D29" s="15">
-        <f>(c_-Rs*SIN($B$29))/COS($B$29)^2</f>
+        <f>(c_-R_sum*SIN($B$29))/COS($B$29)^2</f>
         <v/>
       </c>
     </row>
@@ -2344,11 +2344,11 @@
         <v/>
       </c>
       <c r="C30" s="16">
-        <f>Rs*(1-COS($B$30))+(c_-Rs*SIN($B$30))*TAN($B$30)-H_mid</f>
+        <f>R_sum*(1-COS($B$30))+(c_-R_sum*SIN($B$30))*TAN($B$30)-H_mid</f>
         <v/>
       </c>
       <c r="D30" s="15">
-        <f>(c_-Rs*SIN($B$30))/COS($B$30)^2</f>
+        <f>(c_-R_sum*SIN($B$30))/COS($B$30)^2</f>
         <v/>
       </c>
     </row>
@@ -2361,11 +2361,11 @@
         <v/>
       </c>
       <c r="C31" s="16">
-        <f>Rs*(1-COS($B$31))+(c_-Rs*SIN($B$31))*TAN($B$31)-H_mid</f>
+        <f>R_sum*(1-COS($B$31))+(c_-R_sum*SIN($B$31))*TAN($B$31)-H_mid</f>
         <v/>
       </c>
       <c r="D31" s="15">
-        <f>(c_-Rs*SIN($B$31))/COS($B$31)^2</f>
+        <f>(c_-R_sum*SIN($B$31))/COS($B$31)^2</f>
         <v/>
       </c>
     </row>
@@ -2378,11 +2378,11 @@
         <v/>
       </c>
       <c r="C32" s="16">
-        <f>Rs*(1-COS($B$32))+(c_-Rs*SIN($B$32))*TAN($B$32)-H_mid</f>
+        <f>R_sum*(1-COS($B$32))+(c_-R_sum*SIN($B$32))*TAN($B$32)-H_mid</f>
         <v/>
       </c>
       <c r="D32" s="15">
-        <f>(c_-Rs*SIN($B$32))/COS($B$32)^2</f>
+        <f>(c_-R_sum*SIN($B$32))/COS($B$32)^2</f>
         <v/>
       </c>
     </row>
@@ -2395,11 +2395,11 @@
         <v/>
       </c>
       <c r="C33" s="16">
-        <f>Rs*(1-COS($B$33))+(c_-Rs*SIN($B$33))*TAN($B$33)-H_mid</f>
+        <f>R_sum*(1-COS($B$33))+(c_-R_sum*SIN($B$33))*TAN($B$33)-H_mid</f>
         <v/>
       </c>
       <c r="D33" s="15">
-        <f>(c_-Rs*SIN($B$33))/COS($B$33)^2</f>
+        <f>(c_-R_sum*SIN($B$33))/COS($B$33)^2</f>
         <v/>
       </c>
     </row>
@@ -2412,11 +2412,11 @@
         <v/>
       </c>
       <c r="C34" s="16">
-        <f>Rs*(1-COS($B$34))+(c_-Rs*SIN($B$34))*TAN($B$34)-H_mid</f>
+        <f>R_sum*(1-COS($B$34))+(c_-R_sum*SIN($B$34))*TAN($B$34)-H_mid</f>
         <v/>
       </c>
       <c r="D34" s="15">
-        <f>(c_-Rs*SIN($B$34))/COS($B$34)^2</f>
+        <f>(c_-R_sum*SIN($B$34))/COS($B$34)^2</f>
         <v/>
       </c>
     </row>
@@ -2429,11 +2429,11 @@
         <v/>
       </c>
       <c r="C35" s="16">
-        <f>Rs*(1-COS($B$35))+(c_-Rs*SIN($B$35))*TAN($B$35)-H_mid</f>
+        <f>R_sum*(1-COS($B$35))+(c_-R_sum*SIN($B$35))*TAN($B$35)-H_mid</f>
         <v/>
       </c>
       <c r="D35" s="15">
-        <f>(c_-Rs*SIN($B$35))/COS($B$35)^2</f>
+        <f>(c_-R_sum*SIN($B$35))/COS($B$35)^2</f>
         <v/>
       </c>
     </row>
@@ -2446,11 +2446,11 @@
         <v/>
       </c>
       <c r="C36" s="16">
-        <f>Rs*(1-COS($B$36))+(c_-Rs*SIN($B$36))*TAN($B$36)-H_mid</f>
+        <f>R_sum*(1-COS($B$36))+(c_-R_sum*SIN($B$36))*TAN($B$36)-H_mid</f>
         <v/>
       </c>
       <c r="D36" s="15">
-        <f>(c_-Rs*SIN($B$36))/COS($B$36)^2</f>
+        <f>(c_-R_sum*SIN($B$36))/COS($B$36)^2</f>
         <v/>
       </c>
     </row>
@@ -2463,11 +2463,11 @@
         <v/>
       </c>
       <c r="C37" s="16">
-        <f>Rs*(1-COS($B$37))+(c_-Rs*SIN($B$37))*TAN($B$37)-H_mid</f>
+        <f>R_sum*(1-COS($B$37))+(c_-R_sum*SIN($B$37))*TAN($B$37)-H_mid</f>
         <v/>
       </c>
       <c r="D37" s="15">
-        <f>(c_-Rs*SIN($B$37))/COS($B$37)^2</f>
+        <f>(c_-R_sum*SIN($B$37))/COS($B$37)^2</f>
         <v/>
       </c>
     </row>
@@ -2480,11 +2480,11 @@
         <v/>
       </c>
       <c r="C38" s="16">
-        <f>Rs*(1-COS($B$38))+(c_-Rs*SIN($B$38))*TAN($B$38)-H_mid</f>
+        <f>R_sum*(1-COS($B$38))+(c_-R_sum*SIN($B$38))*TAN($B$38)-H_mid</f>
         <v/>
       </c>
       <c r="D38" s="15">
-        <f>(c_-Rs*SIN($B$38))/COS($B$38)^2</f>
+        <f>(c_-R_sum*SIN($B$38))/COS($B$38)^2</f>
         <v/>
       </c>
     </row>
@@ -2497,11 +2497,11 @@
         <v/>
       </c>
       <c r="C39" s="16">
-        <f>Rs*(1-COS($B$39))+(c_-Rs*SIN($B$39))*TAN($B$39)-H_mid</f>
+        <f>R_sum*(1-COS($B$39))+(c_-R_sum*SIN($B$39))*TAN($B$39)-H_mid</f>
         <v/>
       </c>
       <c r="D39" s="15">
-        <f>(c_-Rs*SIN($B$39))/COS($B$39)^2</f>
+        <f>(c_-R_sum*SIN($B$39))/COS($B$39)^2</f>
         <v/>
       </c>
     </row>
@@ -2514,11 +2514,11 @@
         <v/>
       </c>
       <c r="C40" s="16">
-        <f>Rs*(1-COS($B$40))+(c_-Rs*SIN($B$40))*TAN($B$40)-H_mid</f>
+        <f>R_sum*(1-COS($B$40))+(c_-R_sum*SIN($B$40))*TAN($B$40)-H_mid</f>
         <v/>
       </c>
       <c r="D40" s="15">
-        <f>(c_-Rs*SIN($B$40))/COS($B$40)^2</f>
+        <f>(c_-R_sum*SIN($B$40))/COS($B$40)^2</f>
         <v/>
       </c>
     </row>
@@ -2531,11 +2531,11 @@
         <v/>
       </c>
       <c r="C41" s="16">
-        <f>Rs*(1-COS($B$41))+(c_-Rs*SIN($B$41))*TAN($B$41)-H_mid</f>
+        <f>R_sum*(1-COS($B$41))+(c_-R_sum*SIN($B$41))*TAN($B$41)-H_mid</f>
         <v/>
       </c>
       <c r="D41" s="15">
-        <f>(c_-Rs*SIN($B$41))/COS($B$41)^2</f>
+        <f>(c_-R_sum*SIN($B$41))/COS($B$41)^2</f>
         <v/>
       </c>
     </row>
@@ -2548,11 +2548,11 @@
         <v/>
       </c>
       <c r="C42" s="16">
-        <f>Rs*(1-COS($B$42))+(c_-Rs*SIN($B$42))*TAN($B$42)-H_mid</f>
+        <f>R_sum*(1-COS($B$42))+(c_-R_sum*SIN($B$42))*TAN($B$42)-H_mid</f>
         <v/>
       </c>
       <c r="D42" s="15">
-        <f>(c_-Rs*SIN($B$42))/COS($B$42)^2</f>
+        <f>(c_-R_sum*SIN($B$42))/COS($B$42)^2</f>
         <v/>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="B52" s="8">
-        <f>MAX(0,(c_-(Rc+Rv)*SIN(alpha))/COS(alpha))</f>
+        <f>MAX(0,(c_-(R_crest+R_valley)*SIN(alpha))/COS(alpha))</f>
         <v/>
       </c>
       <c r="C52" s="8" t="inlineStr">
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="B53" s="8">
-        <f>MIN(Rc,Rv)</f>
+        <f>MIN(R_crest,R_valley)</f>
         <v/>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="B54" s="16">
-        <f>(Rc+Rv)*(1-COS(alpha))+TL*SIN(alpha)-H_mid</f>
+        <f>(R_crest+R_valley)*(1-COS(alpha))+TL*SIN(alpha)-H_mid</f>
         <v/>
       </c>
       <c r="C54" s="8" t="inlineStr">
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="B58" s="8">
-        <f>(Rc+Rv)*alpha+TL</f>
+        <f>(R_crest+R_valley)*alpha+TL</f>
         <v/>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="B61" s="8">
-        <f>2*((Rc+Rv)*q_int+TL*COS(alpha)^2)</f>
+        <f>2*((R_crest+R_valley)*q_int+TL*COS(alpha)^2)</f>
         <v/>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="B62" s="8">
-        <f>f_-Rc</f>
+        <f>f_-R_crest</f>
         <v/>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="B63" s="8">
-        <f>f_-Rv</f>
+        <f>f_-R_valley</f>
         <v/>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -2900,7 +2900,7 @@
         </is>
       </c>
       <c r="B64" s="8">
-        <f>f_-Rc*(1-COS(alpha))</f>
+        <f>f_-R_crest*(1-COS(alpha))</f>
         <v/>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -2934,7 +2934,7 @@
         </is>
       </c>
       <c r="B66" s="8">
-        <f>Rc*(a_c^2*alpha+2*a_c*Rc*SIN(alpha)+Rc^2*q_int)</f>
+        <f>R_crest*(a_c^2*alpha+2*a_c*R_crest*SIN(alpha)+R_crest^2*q_int)</f>
         <v/>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="B67" s="8">
-        <f>Rv*(a_v^2*alpha+2*a_v*Rv*SIN(alpha)+Rv^2*q_int)</f>
+        <f>R_valley*(a_v^2*alpha+2*a_v*R_valley*SIN(alpha)+R_valley^2*q_int)</f>
         <v/>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -5095,7 +5095,7 @@
         </is>
       </c>
       <c r="B30" s="16">
-        <f>-(exx+nu_*eyy)/CC</f>
+        <f>-(exx+nu_*eyy)/C_ye</f>
         <v/>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="B32" s="8">
-        <f>1+h_calc^2/(48*Rc^2)</f>
+        <f>1+h_calc^2/(48*R_crest^2)</f>
         <v/>
       </c>
       <c r="C32" s="8" t="inlineStr"/>
@@ -5142,7 +5142,7 @@
         </is>
       </c>
       <c r="B33" s="8">
-        <f>1+h_calc^2/(48*Rv^2)</f>
+        <f>1+h_calc^2/(48*R_valley^2)</f>
         <v/>
       </c>
       <c r="C33" s="8" t="inlineStr"/>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="B34" s="8">
-        <f>2*Rc*alpha/ch_c+2*TL+2*Rv*alpha/ch_v</f>
+        <f>2*R_crest*alpha/ch_c+2*TL+2*R_valley*alpha/ch_v</f>
         <v/>
       </c>
       <c r="C34" s="8" t="inlineStr">
@@ -5296,11 +5296,11 @@
         </is>
       </c>
       <c r="B43" s="16">
-        <f>(c_2+h_calc^2*kxy/(12*Rc))/ch_c</f>
+        <f>(c_2+h_calc^2*kxy/(12*R_crest))/ch_c</f>
         <v/>
       </c>
       <c r="C43" s="16">
-        <f>(c_2-h_calc^2*kxy/(12*Rv))/ch_v</f>
+        <f>(c_2-h_calc^2*kxy/(12*R_valley))/ch_v</f>
         <v/>
       </c>
       <c r="D43" s="10" t="inlineStr">
@@ -5356,11 +5356,11 @@
         </is>
       </c>
       <c r="B46" s="16">
-        <f>(-2*kxy-c_2/(2*Rc))/ch_c</f>
+        <f>(-2*kxy-c_2/(2*R_crest))/ch_c</f>
         <v/>
       </c>
       <c r="C46" s="16">
-        <f>(-2*kxy+c_2/(2*Rv))/ch_v</f>
+        <f>(-2*kxy+c_2/(2*R_valley))/ch_v</f>
         <v/>
       </c>
       <c r="D46" s="10" t="inlineStr">
@@ -5974,7 +5974,7 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>IF(zsgn&gt;0,Rc,Rv)</f>
+        <f>IF(zsgn&gt;0,R_crest,R_valley)</f>
         <v/>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -5995,7 +5995,7 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>IF(zsgn&gt;0,Rv,Rc)</f>
+        <f>IF(zsgn&gt;0,R_valley,R_crest)</f>
         <v/>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>Rc+h_calc/2</f>
+        <f>R_crest+h_calc/2</f>
         <v/>
       </c>
       <c r="C18" s="8" t="inlineStr">

</xml_diff>